<commit_message>
docs: clarify expense mapping and recognition in intake workbook
</commit_message>
<xml_diff>
--- a/outputs/intake-v2/company-intake-v2.xlsx
+++ b/outputs/intake-v2/company-intake-v2.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business" sheetId="1" r:id="R3cc4b31251e14fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly history" sheetId="2" r:id="R25968c5258374e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing expenses" sheetId="3" r:id="Raca997f9e6274885"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opening balances" sheetId="4" r:id="Rc0148147d0ef449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loans" sheetId="5" r:id="Rcd94886d043e41a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="6" r:id="Rbb647d5014c14031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="7" r:id="R5dda51b8c77542b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="8" r:id="Rbdcb87fae9854025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business" sheetId="1" r:id="R0e918c1d240548bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly history" sheetId="2" r:id="R51485f67b6eb431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing expenses" sheetId="3" r:id="R36645dd7069a4838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opening balances" sheetId="4" r:id="R38337f07751b45bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loans" sheetId="5" r:id="Rfac10c006b834e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="6" r:id="R51dc3615715a4b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="7" r:id="Rf8e8f53b821c4214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="8" r:id="Rf9f74aa76021408e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6246,9 +6246,9 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re838fcfb81ae4434"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76ba98ad8ca14664"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61ba4ffef24742c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R938b890a43f44377"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7d59dac9e664a1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7c382acee274f39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13354,7 +13354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2091699c26bf4f4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71dd5458bc0d4da9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14067,7 +14067,9 @@
       <x:c r="S24" s="1"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
-      <x:c r="A25" s="1"/>
+      <x:c r="A25" s="3" t="str">
+        <x:v>How to map existing expenses</x:v>
+      </x:c>
       <x:c r="B25" s="1"/>
       <x:c r="C25" s="1"/>
       <x:c r="D25" s="1"/>
@@ -14088,7 +14090,9 @@
       <x:c r="S25" s="1"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
-      <x:c r="A26" s="1"/>
+      <x:c r="A26" s="1" t="str">
+        <x:v>replace_total: use reconciled item details instead of the category total. Do not add both.</x:v>
+      </x:c>
       <x:c r="B26" s="1"/>
       <x:c r="C26" s="1"/>
       <x:c r="D26" s="1"/>
@@ -14109,7 +14113,9 @@
       <x:c r="S26" s="1"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
-      <x:c r="A27" s="1"/>
+      <x:c r="A27" s="1" t="str">
+        <x:v>included_detail: describe an expense already inside the category total. It adds no extra cost.</x:v>
+      </x:c>
       <x:c r="B27" s="1"/>
       <x:c r="C27" s="1"/>
       <x:c r="D27" s="1"/>
@@ -14130,7 +14136,9 @@
       <x:c r="S27" s="1"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
-      <x:c r="A28" s="1"/>
+      <x:c r="A28" s="1" t="str">
+        <x:v>normalized_recognition_amount is the monthly recognized expense, not the payment.</x:v>
+      </x:c>
       <x:c r="B28" s="1"/>
       <x:c r="C28" s="1"/>
       <x:c r="D28" s="1"/>
@@ -14151,7 +14159,9 @@
       <x:c r="S28" s="1"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
-      <x:c r="A29" s="1"/>
+      <x:c r="A29" s="1" t="str">
+        <x:v>Example: $1,200 annual insurance may be recognized as $100/month where accounting supports it.</x:v>
+      </x:c>
       <x:c r="B29" s="1"/>
       <x:c r="C29" s="1"/>
       <x:c r="D29" s="1"/>
@@ -14172,7 +14182,9 @@
       <x:c r="S29" s="1"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
-      <x:c r="A30" s="1"/>
+      <x:c r="A30" s="1" t="str">
+        <x:v>The $1,200 payment stays a separate source fact. It does not become twelve $100 cash payments.</x:v>
+      </x:c>
       <x:c r="B30" s="1"/>
       <x:c r="C30" s="1"/>
       <x:c r="D30" s="1"/>
@@ -14193,7 +14205,9 @@
       <x:c r="S30" s="1"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
-      <x:c r="A31" s="1"/>
+      <x:c r="A31" s="1" t="str">
+        <x:v>Material irregular payment timing blocks compilation until baseline scheduling is supported.</x:v>
+      </x:c>
       <x:c r="B31" s="1"/>
       <x:c r="C31" s="1"/>
       <x:c r="D31" s="1"/>
@@ -19023,14 +19037,17 @@
       <x:c r="S260" s="1"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D10:D22">
       <x:formula1>"unknown,entered,reviewed_estimate,confirmed,not_applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C16">
+      <x:formula1>"replace_total,included_detail"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R388421efb9184e31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90d7af28a9904a71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24624,7 +24641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac9b595b23d445c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b556dc3d5384387"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30260,7 +30277,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f074791888e4b1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcea0e88b37924e14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35866,7 +35883,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c491350e4841d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8a75e5d2fa440d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41684,12 +41701,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="6">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4903769aed149bf"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R042ee50dea8e4941"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98a1b7ca9a7043f0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc16e2d2ebbd24ea7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33c28bd9fec24ea6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra135e00bb21442b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbf83b451c8543cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e838fe269d4667"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24cb139f4a7d4cee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ae1e4f88c2842b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c8831ec79ae4c8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bbb112155164552"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47467,7 +47484,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cb75db183754244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc202cbfa4836490b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>